<commit_message>
i added magnitude finally
</commit_message>
<xml_diff>
--- a/AI_Tuning_Log.xlsx
+++ b/AI_Tuning_Log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="40">
   <si>
     <t>Parameter</t>
   </si>
@@ -165,7 +165,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -202,6 +202,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9467BD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF8C564B"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -230,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -238,6 +250,8 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1428,6 +1442,676 @@
                 </c:pt>
                 <c:pt idx="49">
                   <c:v>0.6205700502460804</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>…=20 l=2 h=128 lb=60</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="9467BD"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sniper!$A$17:$A$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sniper!$N$17:$N$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>0.6942759476729972</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.6933672900400922</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.6932230588416926</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.693330328583594</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.6936549897564539</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.6937651215940426</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.6937445980146468</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.6937780286242026</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.6937154446254057</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.6936135013910174</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.6934214792729918</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.6930800040160907</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.6926858993853194</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.6922657237671662</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.6915673185726219</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.6907583262143139</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.6899111416385983</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.6888554989210515</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.6876367615159236</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.6863464097415304</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.6853468506888598</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.6839561031871262</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.6826733117286568</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.6804665835532852</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.6787883215688686</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.6767367096527533</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.6751196187543747</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.6731421081677624</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.6703672964572664</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.6682074023594179</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.6658764993209152</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>0.6634242322136096</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0.6610626317541032</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0.6584500991995549</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0.6562485799955924</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0.653986981538202</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>0.6511788974276345</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>0.6488203790203778</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>0.6466857423892359</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>0.6441692327501819</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>0.6419691409697261</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>0.6405149079809218</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>0.6382437429560278</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>0.6360498494518163</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>0.6338576763168225</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>0.6320536120617782</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>0.62992047490878</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>0.6275142644928537</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>0.6258949472466839</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>0.6245671092552562</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:v>…=20 l=2 h=128 lb=60</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="8C564B"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sniper!$A$17:$A$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sniper!$Q$17:$Q$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>0.6975193408128193</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.6936582392275338</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.6932542671214343</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.6933798601801363</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.6937159030936458</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.6937988466116952</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.6938431445036799</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.6938390625022114</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.6938282359379689</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.6937941611956315</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.6936987722156347</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.6935949227596768</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.6934047544966434</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.6931845363903412</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.6931200117898284</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.6927115249000998</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.6925585224518298</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.6919428093621814</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.6914508822483114</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.6903871501664637</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.6900619129654455</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.6892792681600299</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.6882058441355705</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.6873681423984758</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.6861368985245733</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.6850452915385977</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.6838694006046249</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.6823947964833407</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.6806524108374835</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.6792884442949552</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.6777343966217625</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>0.6759341492785023</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0.6740485625036299</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0.6719797017104577</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0.6699965462244214</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0.6685539255220242</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>0.6660743982380565</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>0.6645062510804448</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>0.6627560491467206</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>0.6606335007840268</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>0.6585645881750719</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>0.6569067271948965</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>0.655632032112668</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>0.6531380447382145</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>0.6512039093621207</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>0.6498521883742637</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>0.6482258067766442</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>0.6465681861683119</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>0.6446135454988517</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>0.6427861691070887</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2572,7 +3256,7 @@
                   <c:v>49.25644565245351</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>49.484090577815124</c:v>
+                  <c:v>49.48409057781512</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>49.63808315256068</c:v>
@@ -2608,7 +3292,7 @@
                   <c:v>54.073343679530815</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>54.409623678501916</c:v>
+                  <c:v>54.40962367850192</c:v>
                 </c:pt>
                 <c:pt idx="21">
                   <c:v>54.881633213008776</c:v>
@@ -2696,6 +3380,676 @@
                 </c:pt>
                 <c:pt idx="49">
                   <c:v>64.22930831954316</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>…=20 l=2 h=128 lb=60</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="9467BD"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sniper!$A$17:$A$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sniper!$O$17:$O$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>49.76369184736873</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>49.13382011679403</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>49.38406875037189</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>49.44093571228208</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>49.13620019890686</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>49.14487049803218</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>49.46601157739942</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>49.49635762433804</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>49.78443256292342</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>49.85141487381315</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>50.06222214666406</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>50.24276837550895</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>50.385913314009336</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>50.53798356043283</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>50.980423824621944</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>52.04695561996889</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>52.57269875810715</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>53.19245513970232</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>53.68479212532833</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>54.132332565473504</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>54.50915056569452</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>54.83615684741123</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>55.26482663651896</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>55.81088547554891</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>56.12675637309488</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>56.58424215635439</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>56.861606725432026</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>57.30421699548634</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>57.88597706620878</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>58.17507203998537</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>58.49077293166614</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>58.936443307294105</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>59.32133658611222</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>59.748051307770126</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>60.014280492676995</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>60.385063284683326</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>60.850284334809544</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>61.098917912667986</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>61.479731050721256</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>61.77095109781288</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>61.99858895131882</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>62.21696148517124</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>62.48948088709061</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>62.817677209863746</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>63.11238237719201</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>63.25017213093852</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>63.49744566187534</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>63.78985575002337</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>63.98553250087128</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>64.10139149800668</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:v>…=20 l=2 h=128 lb=60</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="8C564B"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sniper!$A$17:$A$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sniper!$R$17:$R$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>49.75034638695035</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>49.11919961238663</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>49.59657608187483</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>49.593685982166384</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>49.123194750218886</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>49.03691677362869</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>49.16127606402421</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>49.25528930748111</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>49.443060785597105</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>49.562404902969156</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>49.8124835306818</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>50.13829977134211</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>50.24370340776757</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>50.32785631104273</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>50.394923624865065</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>50.55880927892012</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>50.66123781270454</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>50.818238229218906</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>51.24656800659623</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>52.249007590761885</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>52.7136336203599</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>53.05959555604668</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>53.62444004318149</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>53.936315802895194</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>54.41641236622663</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>54.646600307710614</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>55.05027923463359</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>55.49322951641832</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>56.017697610567566</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>56.2298649303401</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>56.53060530588305</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>56.99871645571773</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>57.376469488197344</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>57.738921992808756</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>58.040767406475524</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>58.44963151228717</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>58.80196866791905</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>59.08536844521136</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>59.34785750108379</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>59.697984580468024</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>60.0583120117644</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>60.19253164234166</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>60.37367289171477</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>60.812628035667224</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>61.09194767219469</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>61.223447208928704</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>61.41342876329233</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>61.62908120330152</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>61.903215660940305</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>62.155504364900594</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3969,6 +5323,676 @@
             </c:numRef>
           </c:val>
         </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>…=20 l=2 h=128 lb=60</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="9467BD"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sniper!$A$17:$A$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sniper!$P$17:$P$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>16.198842886</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>15.751187835</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>15.76877458</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>16.20627714</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>15.667719286</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>15.593512421</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>15.80071249</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>16.332568717</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>16.943961795</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>18.738389046</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>18.837717579</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>17.978726132</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>17.845917229</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>19.977000574</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>20.756676631</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>19.781895735</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>21.098832053</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18.389512582</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>17.449479153</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>17.547804432</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>17.493003649</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>17.454503849</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>16.734540153</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>17.686471678</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>18.220199567</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>19.521896363</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>20.296829823</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>19.129360956</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>18.673229586</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>19.118943289</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>20.616682571</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>19.034512786</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>20.064468618</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>19.840505329</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>19.29952142</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>18.999874676</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>19.162202385</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>19.473515827</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>19.480849717</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>18.646938765</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>18.937121625</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>20.063407848</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>20.256636357</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>20.195923105</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>19.790291956</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>20.23474035</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>19.805302762</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>20.146969428</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>19.546213047</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>17.740109965</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:v>…=20 l=2 h=128 lb=60</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="8C564B"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sniper!$A$17:$A$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sniper!$S$17:$S$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>18.687928768</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>19.133708417</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>19.327173519</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>19.51873255</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18.538462687</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>18.961328207</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>19.149237324</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>18.538614416</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>18.819778153</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>19.281306386</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>18.637078445</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>19.896051375</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>20.29501352</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>19.13829012</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>18.753733508</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>19.128886641</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>18.897136094</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>19.15033195</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19.000956368</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19.466477709</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>18.914029047</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>18.876792277</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>18.796405589</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>18.739146967</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>18.564392512</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>19.065687495</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>19.127015917</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>18.705096101</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>19.168757413</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>19.135100558</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>18.361011492</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>19.029248193</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>18.520312047</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>18.792583303</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>19.129739144</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>18.364200036</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>19.156252116</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>19.021148297</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>20.252147361</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>19.193275834</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>18.434585877</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>18.250627422</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>18.251817424</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>17.882744904</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>18.165890505</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>18.508961606</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>17.479083267</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>17.800732854</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>17.998392302</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>17.999392381</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
         <c:marker val="1"/>
         <c:axId val="50030001"/>
         <c:axId val="50030002"/>
@@ -4055,13 +6079,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
+      <xdr:col>27</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
@@ -4085,13 +6109,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
+      <xdr:col>27</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
@@ -4115,13 +6139,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>32</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
+      <xdr:col>27</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>46</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
@@ -4431,7 +6455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M66"/>
+  <dimension ref="A1:S66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.7109375" customWidth="1"/>
@@ -4443,9 +6467,13 @@
     <col min="9" max="10" width="10.7109375" customWidth="1"/>
     <col min="11" max="11" width="13.7109375" customWidth="1"/>
     <col min="12" max="13" width="10.7109375" customWidth="1"/>
+    <col min="14" max="14" width="13.7109375" customWidth="1"/>
+    <col min="15" max="16" width="10.7109375" customWidth="1"/>
+    <col min="17" max="17" width="13.7109375" customWidth="1"/>
+    <col min="18" max="19" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4453,7 +6481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:19">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -4461,7 +6489,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:19">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -4469,7 +6497,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:19">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -4477,7 +6505,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:19">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -4485,7 +6513,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:19">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -4493,7 +6521,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:19">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -4501,7 +6529,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:19">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -4509,7 +6537,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:19">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -4517,7 +6545,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:19">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -4525,7 +6553,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:19">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -4533,7 +6561,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:19">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -4541,7 +6569,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:19">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -4549,7 +6577,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
+    <row r="14" spans="1:19">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -4557,7 +6585,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:19">
       <c r="A15" s="2" t="s">
         <v>26</v>
       </c>
@@ -4573,8 +6601,14 @@
       <c r="E15" s="6" t="s">
         <v>29</v>
       </c>
+      <c r="F15" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:19">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
@@ -4614,8 +6648,26 @@
       <c r="M16" s="1" t="s">
         <v>39</v>
       </c>
+      <c r="N16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="P16" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="S16" s="1" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:19">
       <c r="A17">
         <v>1</v>
       </c>
@@ -4655,8 +6707,26 @@
       <c r="M17">
         <v>16.807420029</v>
       </c>
+      <c r="N17">
+        <v>0.6942759476729972</v>
+      </c>
+      <c r="O17">
+        <v>49.76369184736873</v>
+      </c>
+      <c r="P17">
+        <v>16.198842886</v>
+      </c>
+      <c r="Q17">
+        <v>0.6975193408128193</v>
+      </c>
+      <c r="R17">
+        <v>49.75034638695035</v>
+      </c>
+      <c r="S17">
+        <v>18.687928768</v>
+      </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:19">
       <c r="A18">
         <v>2</v>
       </c>
@@ -4696,8 +6766,26 @@
       <c r="M18">
         <v>16.745763815</v>
       </c>
+      <c r="N18">
+        <v>0.6933672900400922</v>
+      </c>
+      <c r="O18">
+        <v>49.13382011679403</v>
+      </c>
+      <c r="P18">
+        <v>15.751187835</v>
+      </c>
+      <c r="Q18">
+        <v>0.6936582392275338</v>
+      </c>
+      <c r="R18">
+        <v>49.11919961238663</v>
+      </c>
+      <c r="S18">
+        <v>19.133708417</v>
+      </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:19">
       <c r="A19">
         <v>3</v>
       </c>
@@ -4737,8 +6825,26 @@
       <c r="M19">
         <v>16.7762943</v>
       </c>
+      <c r="N19">
+        <v>0.6932230588416926</v>
+      </c>
+      <c r="O19">
+        <v>49.38406875037189</v>
+      </c>
+      <c r="P19">
+        <v>15.76877458</v>
+      </c>
+      <c r="Q19">
+        <v>0.6932542671214343</v>
+      </c>
+      <c r="R19">
+        <v>49.59657608187483</v>
+      </c>
+      <c r="S19">
+        <v>19.327173519</v>
+      </c>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:19">
       <c r="A20">
         <v>4</v>
       </c>
@@ -4778,8 +6884,26 @@
       <c r="M20">
         <v>16.62535558</v>
       </c>
+      <c r="N20">
+        <v>0.693330328583594</v>
+      </c>
+      <c r="O20">
+        <v>49.44093571228208</v>
+      </c>
+      <c r="P20">
+        <v>16.20627714</v>
+      </c>
+      <c r="Q20">
+        <v>0.6933798601801363</v>
+      </c>
+      <c r="R20">
+        <v>49.593685982166384</v>
+      </c>
+      <c r="S20">
+        <v>19.51873255</v>
+      </c>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:19">
       <c r="A21">
         <v>5</v>
       </c>
@@ -4819,8 +6943,26 @@
       <c r="M21">
         <v>17.285882021</v>
       </c>
+      <c r="N21">
+        <v>0.6936549897564539</v>
+      </c>
+      <c r="O21">
+        <v>49.13620019890686</v>
+      </c>
+      <c r="P21">
+        <v>15.667719286</v>
+      </c>
+      <c r="Q21">
+        <v>0.6937159030936458</v>
+      </c>
+      <c r="R21">
+        <v>49.123194750218886</v>
+      </c>
+      <c r="S21">
+        <v>18.538462687</v>
+      </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:19">
       <c r="A22">
         <v>6</v>
       </c>
@@ -4860,8 +7002,26 @@
       <c r="M22">
         <v>16.871972433</v>
       </c>
+      <c r="N22">
+        <v>0.6937651215940426</v>
+      </c>
+      <c r="O22">
+        <v>49.14487049803218</v>
+      </c>
+      <c r="P22">
+        <v>15.593512421</v>
+      </c>
+      <c r="Q22">
+        <v>0.6937988466116952</v>
+      </c>
+      <c r="R22">
+        <v>49.03691677362869</v>
+      </c>
+      <c r="S22">
+        <v>18.961328207</v>
+      </c>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:19">
       <c r="A23">
         <v>7</v>
       </c>
@@ -4901,8 +7061,26 @@
       <c r="M23">
         <v>16.484371066</v>
       </c>
+      <c r="N23">
+        <v>0.6937445980146468</v>
+      </c>
+      <c r="O23">
+        <v>49.46601157739942</v>
+      </c>
+      <c r="P23">
+        <v>15.80071249</v>
+      </c>
+      <c r="Q23">
+        <v>0.6938431445036799</v>
+      </c>
+      <c r="R23">
+        <v>49.16127606402421</v>
+      </c>
+      <c r="S23">
+        <v>19.149237324</v>
+      </c>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:19">
       <c r="A24">
         <v>8</v>
       </c>
@@ -4942,8 +7120,26 @@
       <c r="M24">
         <v>16.657029986</v>
       </c>
+      <c r="N24">
+        <v>0.6937780286242026</v>
+      </c>
+      <c r="O24">
+        <v>49.49635762433804</v>
+      </c>
+      <c r="P24">
+        <v>16.332568717</v>
+      </c>
+      <c r="Q24">
+        <v>0.6938390625022114</v>
+      </c>
+      <c r="R24">
+        <v>49.25528930748111</v>
+      </c>
+      <c r="S24">
+        <v>18.538614416</v>
+      </c>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:19">
       <c r="A25">
         <v>9</v>
       </c>
@@ -4978,13 +7174,31 @@
         <v>0.6937894375318441</v>
       </c>
       <c r="L25">
-        <v>49.484090577815124</v>
+        <v>49.48409057781512</v>
       </c>
       <c r="M25">
         <v>16.837887456</v>
       </c>
+      <c r="N25">
+        <v>0.6937154446254057</v>
+      </c>
+      <c r="O25">
+        <v>49.78443256292342</v>
+      </c>
+      <c r="P25">
+        <v>16.943961795</v>
+      </c>
+      <c r="Q25">
+        <v>0.6938282359379689</v>
+      </c>
+      <c r="R25">
+        <v>49.443060785597105</v>
+      </c>
+      <c r="S25">
+        <v>18.819778153</v>
+      </c>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:19">
       <c r="A26">
         <v>10</v>
       </c>
@@ -5024,8 +7238,26 @@
       <c r="M26">
         <v>17.12346488</v>
       </c>
+      <c r="N26">
+        <v>0.6936135013910174</v>
+      </c>
+      <c r="O26">
+        <v>49.85141487381315</v>
+      </c>
+      <c r="P26">
+        <v>18.738389046</v>
+      </c>
+      <c r="Q26">
+        <v>0.6937941611956315</v>
+      </c>
+      <c r="R26">
+        <v>49.562404902969156</v>
+      </c>
+      <c r="S26">
+        <v>19.281306386</v>
+      </c>
     </row>
-    <row r="27" spans="1:13">
+    <row r="27" spans="1:19">
       <c r="A27">
         <v>11</v>
       </c>
@@ -5056,8 +7288,26 @@
       <c r="M27">
         <v>16.413742337</v>
       </c>
+      <c r="N27">
+        <v>0.6934214792729918</v>
+      </c>
+      <c r="O27">
+        <v>50.06222214666406</v>
+      </c>
+      <c r="P27">
+        <v>18.837717579</v>
+      </c>
+      <c r="Q27">
+        <v>0.6936987722156347</v>
+      </c>
+      <c r="R27">
+        <v>49.8124835306818</v>
+      </c>
+      <c r="S27">
+        <v>18.637078445</v>
+      </c>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:19">
       <c r="A28">
         <v>12</v>
       </c>
@@ -5088,8 +7338,26 @@
       <c r="M28">
         <v>16.556402943</v>
       </c>
+      <c r="N28">
+        <v>0.6930800040160907</v>
+      </c>
+      <c r="O28">
+        <v>50.24276837550895</v>
+      </c>
+      <c r="P28">
+        <v>17.978726132</v>
+      </c>
+      <c r="Q28">
+        <v>0.6935949227596768</v>
+      </c>
+      <c r="R28">
+        <v>50.13829977134211</v>
+      </c>
+      <c r="S28">
+        <v>19.896051375</v>
+      </c>
     </row>
-    <row r="29" spans="1:13">
+    <row r="29" spans="1:19">
       <c r="A29">
         <v>13</v>
       </c>
@@ -5120,8 +7388,26 @@
       <c r="M29">
         <v>16.514506949</v>
       </c>
+      <c r="N29">
+        <v>0.6926858993853194</v>
+      </c>
+      <c r="O29">
+        <v>50.385913314009336</v>
+      </c>
+      <c r="P29">
+        <v>17.845917229</v>
+      </c>
+      <c r="Q29">
+        <v>0.6934047544966434</v>
+      </c>
+      <c r="R29">
+        <v>50.24370340776757</v>
+      </c>
+      <c r="S29">
+        <v>20.29501352</v>
+      </c>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:19">
       <c r="A30">
         <v>14</v>
       </c>
@@ -5152,8 +7438,26 @@
       <c r="M30">
         <v>16.778240012</v>
       </c>
+      <c r="N30">
+        <v>0.6922657237671662</v>
+      </c>
+      <c r="O30">
+        <v>50.53798356043283</v>
+      </c>
+      <c r="P30">
+        <v>19.977000574</v>
+      </c>
+      <c r="Q30">
+        <v>0.6931845363903412</v>
+      </c>
+      <c r="R30">
+        <v>50.32785631104273</v>
+      </c>
+      <c r="S30">
+        <v>19.13829012</v>
+      </c>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:19">
       <c r="A31">
         <v>15</v>
       </c>
@@ -5184,8 +7488,26 @@
       <c r="M31">
         <v>16.909606975</v>
       </c>
+      <c r="N31">
+        <v>0.6915673185726219</v>
+      </c>
+      <c r="O31">
+        <v>50.980423824621944</v>
+      </c>
+      <c r="P31">
+        <v>20.756676631</v>
+      </c>
+      <c r="Q31">
+        <v>0.6931200117898284</v>
+      </c>
+      <c r="R31">
+        <v>50.394923624865065</v>
+      </c>
+      <c r="S31">
+        <v>18.753733508</v>
+      </c>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:19">
       <c r="A32">
         <v>16</v>
       </c>
@@ -5216,8 +7538,26 @@
       <c r="M32">
         <v>16.586320177</v>
       </c>
+      <c r="N32">
+        <v>0.6907583262143139</v>
+      </c>
+      <c r="O32">
+        <v>52.04695561996889</v>
+      </c>
+      <c r="P32">
+        <v>19.781895735</v>
+      </c>
+      <c r="Q32">
+        <v>0.6927115249000998</v>
+      </c>
+      <c r="R32">
+        <v>50.55880927892012</v>
+      </c>
+      <c r="S32">
+        <v>19.128886641</v>
+      </c>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:19">
       <c r="A33">
         <v>17</v>
       </c>
@@ -5248,8 +7588,26 @@
       <c r="M33">
         <v>16.865581987</v>
       </c>
+      <c r="N33">
+        <v>0.6899111416385983</v>
+      </c>
+      <c r="O33">
+        <v>52.57269875810715</v>
+      </c>
+      <c r="P33">
+        <v>21.098832053</v>
+      </c>
+      <c r="Q33">
+        <v>0.6925585224518298</v>
+      </c>
+      <c r="R33">
+        <v>50.66123781270454</v>
+      </c>
+      <c r="S33">
+        <v>18.897136094</v>
+      </c>
     </row>
-    <row r="34" spans="1:13">
+    <row r="34" spans="1:19">
       <c r="A34">
         <v>18</v>
       </c>
@@ -5280,8 +7638,26 @@
       <c r="M34">
         <v>17.071334063</v>
       </c>
+      <c r="N34">
+        <v>0.6888554989210515</v>
+      </c>
+      <c r="O34">
+        <v>53.19245513970232</v>
+      </c>
+      <c r="P34">
+        <v>18.389512582</v>
+      </c>
+      <c r="Q34">
+        <v>0.6919428093621814</v>
+      </c>
+      <c r="R34">
+        <v>50.818238229218906</v>
+      </c>
+      <c r="S34">
+        <v>19.15033195</v>
+      </c>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:19">
       <c r="A35">
         <v>19</v>
       </c>
@@ -5312,8 +7688,26 @@
       <c r="M35">
         <v>16.870781324</v>
       </c>
+      <c r="N35">
+        <v>0.6876367615159236</v>
+      </c>
+      <c r="O35">
+        <v>53.68479212532833</v>
+      </c>
+      <c r="P35">
+        <v>17.449479153</v>
+      </c>
+      <c r="Q35">
+        <v>0.6914508822483114</v>
+      </c>
+      <c r="R35">
+        <v>51.24656800659623</v>
+      </c>
+      <c r="S35">
+        <v>19.000956368</v>
+      </c>
     </row>
-    <row r="36" spans="1:13">
+    <row r="36" spans="1:19">
       <c r="A36">
         <v>20</v>
       </c>
@@ -5344,8 +7738,26 @@
       <c r="M36">
         <v>17.220750256</v>
       </c>
+      <c r="N36">
+        <v>0.6863464097415304</v>
+      </c>
+      <c r="O36">
+        <v>54.132332565473504</v>
+      </c>
+      <c r="P36">
+        <v>17.547804432</v>
+      </c>
+      <c r="Q36">
+        <v>0.6903871501664637</v>
+      </c>
+      <c r="R36">
+        <v>52.249007590761885</v>
+      </c>
+      <c r="S36">
+        <v>19.466477709</v>
+      </c>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:19">
       <c r="A37">
         <v>21</v>
       </c>
@@ -5371,13 +7783,31 @@
         <v>0.684780174692096</v>
       </c>
       <c r="L37">
-        <v>54.409623678501916</v>
+        <v>54.40962367850192</v>
       </c>
       <c r="M37">
         <v>16.556888934</v>
       </c>
+      <c r="N37">
+        <v>0.6853468506888598</v>
+      </c>
+      <c r="O37">
+        <v>54.50915056569452</v>
+      </c>
+      <c r="P37">
+        <v>17.493003649</v>
+      </c>
+      <c r="Q37">
+        <v>0.6900619129654455</v>
+      </c>
+      <c r="R37">
+        <v>52.7136336203599</v>
+      </c>
+      <c r="S37">
+        <v>18.914029047</v>
+      </c>
     </row>
-    <row r="38" spans="1:13">
+    <row r="38" spans="1:19">
       <c r="A38">
         <v>22</v>
       </c>
@@ -5408,8 +7838,26 @@
       <c r="M38">
         <v>16.717710365</v>
       </c>
+      <c r="N38">
+        <v>0.6839561031871262</v>
+      </c>
+      <c r="O38">
+        <v>54.83615684741123</v>
+      </c>
+      <c r="P38">
+        <v>17.454503849</v>
+      </c>
+      <c r="Q38">
+        <v>0.6892792681600299</v>
+      </c>
+      <c r="R38">
+        <v>53.05959555604668</v>
+      </c>
+      <c r="S38">
+        <v>18.876792277</v>
+      </c>
     </row>
-    <row r="39" spans="1:13">
+    <row r="39" spans="1:19">
       <c r="A39">
         <v>23</v>
       </c>
@@ -5440,8 +7888,26 @@
       <c r="M39">
         <v>16.751196244</v>
       </c>
+      <c r="N39">
+        <v>0.6826733117286568</v>
+      </c>
+      <c r="O39">
+        <v>55.26482663651896</v>
+      </c>
+      <c r="P39">
+        <v>16.734540153</v>
+      </c>
+      <c r="Q39">
+        <v>0.6882058441355705</v>
+      </c>
+      <c r="R39">
+        <v>53.62444004318149</v>
+      </c>
+      <c r="S39">
+        <v>18.796405589</v>
+      </c>
     </row>
-    <row r="40" spans="1:13">
+    <row r="40" spans="1:19">
       <c r="A40">
         <v>24</v>
       </c>
@@ -5472,8 +7938,26 @@
       <c r="M40">
         <v>17.033199997</v>
       </c>
+      <c r="N40">
+        <v>0.6804665835532852</v>
+      </c>
+      <c r="O40">
+        <v>55.81088547554891</v>
+      </c>
+      <c r="P40">
+        <v>17.686471678</v>
+      </c>
+      <c r="Q40">
+        <v>0.6873681423984758</v>
+      </c>
+      <c r="R40">
+        <v>53.936315802895194</v>
+      </c>
+      <c r="S40">
+        <v>18.739146967</v>
+      </c>
     </row>
-    <row r="41" spans="1:13">
+    <row r="41" spans="1:19">
       <c r="A41">
         <v>25</v>
       </c>
@@ -5504,8 +7988,26 @@
       <c r="M41">
         <v>16.795754364</v>
       </c>
+      <c r="N41">
+        <v>0.6787883215688686</v>
+      </c>
+      <c r="O41">
+        <v>56.12675637309488</v>
+      </c>
+      <c r="P41">
+        <v>18.220199567</v>
+      </c>
+      <c r="Q41">
+        <v>0.6861368985245733</v>
+      </c>
+      <c r="R41">
+        <v>54.41641236622663</v>
+      </c>
+      <c r="S41">
+        <v>18.564392512</v>
+      </c>
     </row>
-    <row r="42" spans="1:13">
+    <row r="42" spans="1:19">
       <c r="A42">
         <v>26</v>
       </c>
@@ -5536,8 +8038,26 @@
       <c r="M42">
         <v>16.983905376</v>
       </c>
+      <c r="N42">
+        <v>0.6767367096527533</v>
+      </c>
+      <c r="O42">
+        <v>56.58424215635439</v>
+      </c>
+      <c r="P42">
+        <v>19.521896363</v>
+      </c>
+      <c r="Q42">
+        <v>0.6850452915385977</v>
+      </c>
+      <c r="R42">
+        <v>54.646600307710614</v>
+      </c>
+      <c r="S42">
+        <v>19.065687495</v>
+      </c>
     </row>
-    <row r="43" spans="1:13">
+    <row r="43" spans="1:19">
       <c r="A43">
         <v>27</v>
       </c>
@@ -5568,8 +8088,26 @@
       <c r="M43">
         <v>16.880966869</v>
       </c>
+      <c r="N43">
+        <v>0.6751196187543747</v>
+      </c>
+      <c r="O43">
+        <v>56.861606725432026</v>
+      </c>
+      <c r="P43">
+        <v>20.296829823</v>
+      </c>
+      <c r="Q43">
+        <v>0.6838694006046249</v>
+      </c>
+      <c r="R43">
+        <v>55.05027923463359</v>
+      </c>
+      <c r="S43">
+        <v>19.127015917</v>
+      </c>
     </row>
-    <row r="44" spans="1:13">
+    <row r="44" spans="1:19">
       <c r="A44">
         <v>28</v>
       </c>
@@ -5600,8 +8138,26 @@
       <c r="M44">
         <v>17.142872044</v>
       </c>
+      <c r="N44">
+        <v>0.6731421081677624</v>
+      </c>
+      <c r="O44">
+        <v>57.30421699548634</v>
+      </c>
+      <c r="P44">
+        <v>19.129360956</v>
+      </c>
+      <c r="Q44">
+        <v>0.6823947964833407</v>
+      </c>
+      <c r="R44">
+        <v>55.49322951641832</v>
+      </c>
+      <c r="S44">
+        <v>18.705096101</v>
+      </c>
     </row>
-    <row r="45" spans="1:13">
+    <row r="45" spans="1:19">
       <c r="A45">
         <v>29</v>
       </c>
@@ -5632,8 +8188,26 @@
       <c r="M45">
         <v>16.428273928</v>
       </c>
+      <c r="N45">
+        <v>0.6703672964572664</v>
+      </c>
+      <c r="O45">
+        <v>57.88597706620878</v>
+      </c>
+      <c r="P45">
+        <v>18.673229586</v>
+      </c>
+      <c r="Q45">
+        <v>0.6806524108374835</v>
+      </c>
+      <c r="R45">
+        <v>56.017697610567566</v>
+      </c>
+      <c r="S45">
+        <v>19.168757413</v>
+      </c>
     </row>
-    <row r="46" spans="1:13">
+    <row r="46" spans="1:19">
       <c r="A46">
         <v>30</v>
       </c>
@@ -5664,8 +8238,26 @@
       <c r="M46">
         <v>16.831818185</v>
       </c>
+      <c r="N46">
+        <v>0.6682074023594179</v>
+      </c>
+      <c r="O46">
+        <v>58.17507203998537</v>
+      </c>
+      <c r="P46">
+        <v>19.118943289</v>
+      </c>
+      <c r="Q46">
+        <v>0.6792884442949552</v>
+      </c>
+      <c r="R46">
+        <v>56.2298649303401</v>
+      </c>
+      <c r="S46">
+        <v>19.135100558</v>
+      </c>
     </row>
-    <row r="47" spans="1:13">
+    <row r="47" spans="1:19">
       <c r="A47">
         <v>31</v>
       </c>
@@ -5687,8 +8279,26 @@
       <c r="M47">
         <v>17.643509045</v>
       </c>
+      <c r="N47">
+        <v>0.6658764993209152</v>
+      </c>
+      <c r="O47">
+        <v>58.49077293166614</v>
+      </c>
+      <c r="P47">
+        <v>20.616682571</v>
+      </c>
+      <c r="Q47">
+        <v>0.6777343966217625</v>
+      </c>
+      <c r="R47">
+        <v>56.53060530588305</v>
+      </c>
+      <c r="S47">
+        <v>18.361011492</v>
+      </c>
     </row>
-    <row r="48" spans="1:13">
+    <row r="48" spans="1:19">
       <c r="A48">
         <v>32</v>
       </c>
@@ -5710,8 +8320,26 @@
       <c r="M48">
         <v>18.646936417</v>
       </c>
+      <c r="N48">
+        <v>0.6634242322136096</v>
+      </c>
+      <c r="O48">
+        <v>58.936443307294105</v>
+      </c>
+      <c r="P48">
+        <v>19.034512786</v>
+      </c>
+      <c r="Q48">
+        <v>0.6759341492785023</v>
+      </c>
+      <c r="R48">
+        <v>56.99871645571773</v>
+      </c>
+      <c r="S48">
+        <v>19.029248193</v>
+      </c>
     </row>
-    <row r="49" spans="1:13">
+    <row r="49" spans="1:19">
       <c r="A49">
         <v>33</v>
       </c>
@@ -5733,8 +8361,26 @@
       <c r="M49">
         <v>18.448425695</v>
       </c>
+      <c r="N49">
+        <v>0.6610626317541032</v>
+      </c>
+      <c r="O49">
+        <v>59.32133658611222</v>
+      </c>
+      <c r="P49">
+        <v>20.064468618</v>
+      </c>
+      <c r="Q49">
+        <v>0.6740485625036299</v>
+      </c>
+      <c r="R49">
+        <v>57.376469488197344</v>
+      </c>
+      <c r="S49">
+        <v>18.520312047</v>
+      </c>
     </row>
-    <row r="50" spans="1:13">
+    <row r="50" spans="1:19">
       <c r="A50">
         <v>34</v>
       </c>
@@ -5756,8 +8402,26 @@
       <c r="M50">
         <v>18.610269665</v>
       </c>
+      <c r="N50">
+        <v>0.6584500991995549</v>
+      </c>
+      <c r="O50">
+        <v>59.748051307770126</v>
+      </c>
+      <c r="P50">
+        <v>19.840505329</v>
+      </c>
+      <c r="Q50">
+        <v>0.6719797017104577</v>
+      </c>
+      <c r="R50">
+        <v>57.738921992808756</v>
+      </c>
+      <c r="S50">
+        <v>18.792583303</v>
+      </c>
     </row>
-    <row r="51" spans="1:13">
+    <row r="51" spans="1:19">
       <c r="A51">
         <v>35</v>
       </c>
@@ -5779,8 +8443,26 @@
       <c r="M51">
         <v>18.386114816</v>
       </c>
+      <c r="N51">
+        <v>0.6562485799955924</v>
+      </c>
+      <c r="O51">
+        <v>60.014280492676995</v>
+      </c>
+      <c r="P51">
+        <v>19.29952142</v>
+      </c>
+      <c r="Q51">
+        <v>0.6699965462244214</v>
+      </c>
+      <c r="R51">
+        <v>58.040767406475524</v>
+      </c>
+      <c r="S51">
+        <v>19.129739144</v>
+      </c>
     </row>
-    <row r="52" spans="1:13">
+    <row r="52" spans="1:19">
       <c r="A52">
         <v>36</v>
       </c>
@@ -5802,8 +8484,26 @@
       <c r="M52">
         <v>17.84284724</v>
       </c>
+      <c r="N52">
+        <v>0.653986981538202</v>
+      </c>
+      <c r="O52">
+        <v>60.385063284683326</v>
+      </c>
+      <c r="P52">
+        <v>18.999874676</v>
+      </c>
+      <c r="Q52">
+        <v>0.6685539255220242</v>
+      </c>
+      <c r="R52">
+        <v>58.44963151228717</v>
+      </c>
+      <c r="S52">
+        <v>18.364200036</v>
+      </c>
     </row>
-    <row r="53" spans="1:13">
+    <row r="53" spans="1:19">
       <c r="A53">
         <v>37</v>
       </c>
@@ -5825,8 +8525,26 @@
       <c r="M53">
         <v>17.990654347</v>
       </c>
+      <c r="N53">
+        <v>0.6511788974276345</v>
+      </c>
+      <c r="O53">
+        <v>60.850284334809544</v>
+      </c>
+      <c r="P53">
+        <v>19.162202385</v>
+      </c>
+      <c r="Q53">
+        <v>0.6660743982380565</v>
+      </c>
+      <c r="R53">
+        <v>58.80196866791905</v>
+      </c>
+      <c r="S53">
+        <v>19.156252116</v>
+      </c>
     </row>
-    <row r="54" spans="1:13">
+    <row r="54" spans="1:19">
       <c r="A54">
         <v>38</v>
       </c>
@@ -5848,8 +8566,26 @@
       <c r="M54">
         <v>18.377255822</v>
       </c>
+      <c r="N54">
+        <v>0.6488203790203778</v>
+      </c>
+      <c r="O54">
+        <v>61.098917912667986</v>
+      </c>
+      <c r="P54">
+        <v>19.473515827</v>
+      </c>
+      <c r="Q54">
+        <v>0.6645062510804448</v>
+      </c>
+      <c r="R54">
+        <v>59.08536844521136</v>
+      </c>
+      <c r="S54">
+        <v>19.021148297</v>
+      </c>
     </row>
-    <row r="55" spans="1:13">
+    <row r="55" spans="1:19">
       <c r="A55">
         <v>39</v>
       </c>
@@ -5871,8 +8607,26 @@
       <c r="M55">
         <v>18.66298113</v>
       </c>
+      <c r="N55">
+        <v>0.6466857423892359</v>
+      </c>
+      <c r="O55">
+        <v>61.479731050721256</v>
+      </c>
+      <c r="P55">
+        <v>19.480849717</v>
+      </c>
+      <c r="Q55">
+        <v>0.6627560491467206</v>
+      </c>
+      <c r="R55">
+        <v>59.34785750108379</v>
+      </c>
+      <c r="S55">
+        <v>20.252147361</v>
+      </c>
     </row>
-    <row r="56" spans="1:13">
+    <row r="56" spans="1:19">
       <c r="A56">
         <v>40</v>
       </c>
@@ -5894,8 +8648,26 @@
       <c r="M56">
         <v>18.63036799</v>
       </c>
+      <c r="N56">
+        <v>0.6441692327501819</v>
+      </c>
+      <c r="O56">
+        <v>61.77095109781288</v>
+      </c>
+      <c r="P56">
+        <v>18.646938765</v>
+      </c>
+      <c r="Q56">
+        <v>0.6606335007840268</v>
+      </c>
+      <c r="R56">
+        <v>59.697984580468024</v>
+      </c>
+      <c r="S56">
+        <v>19.193275834</v>
+      </c>
     </row>
-    <row r="57" spans="1:13">
+    <row r="57" spans="1:19">
       <c r="A57">
         <v>41</v>
       </c>
@@ -5917,8 +8689,26 @@
       <c r="M57">
         <v>18.22543177</v>
       </c>
+      <c r="N57">
+        <v>0.6419691409697261</v>
+      </c>
+      <c r="O57">
+        <v>61.99858895131882</v>
+      </c>
+      <c r="P57">
+        <v>18.937121625</v>
+      </c>
+      <c r="Q57">
+        <v>0.6585645881750719</v>
+      </c>
+      <c r="R57">
+        <v>60.0583120117644</v>
+      </c>
+      <c r="S57">
+        <v>18.434585877</v>
+      </c>
     </row>
-    <row r="58" spans="1:13">
+    <row r="58" spans="1:19">
       <c r="A58">
         <v>42</v>
       </c>
@@ -5940,8 +8730,26 @@
       <c r="M58">
         <v>18.381927043</v>
       </c>
+      <c r="N58">
+        <v>0.6405149079809218</v>
+      </c>
+      <c r="O58">
+        <v>62.21696148517124</v>
+      </c>
+      <c r="P58">
+        <v>20.063407848</v>
+      </c>
+      <c r="Q58">
+        <v>0.6569067271948965</v>
+      </c>
+      <c r="R58">
+        <v>60.19253164234166</v>
+      </c>
+      <c r="S58">
+        <v>18.250627422</v>
+      </c>
     </row>
-    <row r="59" spans="1:13">
+    <row r="59" spans="1:19">
       <c r="A59">
         <v>43</v>
       </c>
@@ -5963,8 +8771,26 @@
       <c r="M59">
         <v>18.261934743</v>
       </c>
+      <c r="N59">
+        <v>0.6382437429560278</v>
+      </c>
+      <c r="O59">
+        <v>62.48948088709061</v>
+      </c>
+      <c r="P59">
+        <v>20.256636357</v>
+      </c>
+      <c r="Q59">
+        <v>0.655632032112668</v>
+      </c>
+      <c r="R59">
+        <v>60.37367289171477</v>
+      </c>
+      <c r="S59">
+        <v>18.251817424</v>
+      </c>
     </row>
-    <row r="60" spans="1:13">
+    <row r="60" spans="1:19">
       <c r="A60">
         <v>44</v>
       </c>
@@ -5986,8 +8812,26 @@
       <c r="M60">
         <v>18.46606709</v>
       </c>
+      <c r="N60">
+        <v>0.6360498494518163</v>
+      </c>
+      <c r="O60">
+        <v>62.817677209863746</v>
+      </c>
+      <c r="P60">
+        <v>20.195923105</v>
+      </c>
+      <c r="Q60">
+        <v>0.6531380447382145</v>
+      </c>
+      <c r="R60">
+        <v>60.812628035667224</v>
+      </c>
+      <c r="S60">
+        <v>17.882744904</v>
+      </c>
     </row>
-    <row r="61" spans="1:13">
+    <row r="61" spans="1:19">
       <c r="A61">
         <v>45</v>
       </c>
@@ -6009,8 +8853,26 @@
       <c r="M61">
         <v>17.896320977</v>
       </c>
+      <c r="N61">
+        <v>0.6338576763168225</v>
+      </c>
+      <c r="O61">
+        <v>63.11238237719201</v>
+      </c>
+      <c r="P61">
+        <v>19.790291956</v>
+      </c>
+      <c r="Q61">
+        <v>0.6512039093621207</v>
+      </c>
+      <c r="R61">
+        <v>61.09194767219469</v>
+      </c>
+      <c r="S61">
+        <v>18.165890505</v>
+      </c>
     </row>
-    <row r="62" spans="1:13">
+    <row r="62" spans="1:19">
       <c r="A62">
         <v>46</v>
       </c>
@@ -6032,8 +8894,26 @@
       <c r="M62">
         <v>18.783552359</v>
       </c>
+      <c r="N62">
+        <v>0.6320536120617782</v>
+      </c>
+      <c r="O62">
+        <v>63.25017213093852</v>
+      </c>
+      <c r="P62">
+        <v>20.23474035</v>
+      </c>
+      <c r="Q62">
+        <v>0.6498521883742637</v>
+      </c>
+      <c r="R62">
+        <v>61.223447208928704</v>
+      </c>
+      <c r="S62">
+        <v>18.508961606</v>
+      </c>
     </row>
-    <row r="63" spans="1:13">
+    <row r="63" spans="1:19">
       <c r="A63">
         <v>47</v>
       </c>
@@ -6055,8 +8935,26 @@
       <c r="M63">
         <v>18.171472017</v>
       </c>
+      <c r="N63">
+        <v>0.62992047490878</v>
+      </c>
+      <c r="O63">
+        <v>63.49744566187534</v>
+      </c>
+      <c r="P63">
+        <v>19.805302762</v>
+      </c>
+      <c r="Q63">
+        <v>0.6482258067766442</v>
+      </c>
+      <c r="R63">
+        <v>61.41342876329233</v>
+      </c>
+      <c r="S63">
+        <v>17.479083267</v>
+      </c>
     </row>
-    <row r="64" spans="1:13">
+    <row r="64" spans="1:19">
       <c r="A64">
         <v>48</v>
       </c>
@@ -6078,8 +8976,26 @@
       <c r="M64">
         <v>18.240496971</v>
       </c>
+      <c r="N64">
+        <v>0.6275142644928537</v>
+      </c>
+      <c r="O64">
+        <v>63.78985575002337</v>
+      </c>
+      <c r="P64">
+        <v>20.146969428</v>
+      </c>
+      <c r="Q64">
+        <v>0.6465681861683119</v>
+      </c>
+      <c r="R64">
+        <v>61.62908120330152</v>
+      </c>
+      <c r="S64">
+        <v>17.800732854</v>
+      </c>
     </row>
-    <row r="65" spans="1:13">
+    <row r="65" spans="1:19">
       <c r="A65">
         <v>49</v>
       </c>
@@ -6101,8 +9017,26 @@
       <c r="M65">
         <v>18.675442032</v>
       </c>
+      <c r="N65">
+        <v>0.6258949472466839</v>
+      </c>
+      <c r="O65">
+        <v>63.98553250087128</v>
+      </c>
+      <c r="P65">
+        <v>19.546213047</v>
+      </c>
+      <c r="Q65">
+        <v>0.6446135454988517</v>
+      </c>
+      <c r="R65">
+        <v>61.903215660940305</v>
+      </c>
+      <c r="S65">
+        <v>17.998392302</v>
+      </c>
     </row>
-    <row r="66" spans="1:13">
+    <row r="66" spans="1:19">
       <c r="A66">
         <v>50</v>
       </c>
@@ -6123,6 +9057,24 @@
       </c>
       <c r="M66">
         <v>17.9649802</v>
+      </c>
+      <c r="N66">
+        <v>0.6245671092552562</v>
+      </c>
+      <c r="O66">
+        <v>64.10139149800668</v>
+      </c>
+      <c r="P66">
+        <v>17.740109965</v>
+      </c>
+      <c r="Q66">
+        <v>0.6427861691070887</v>
+      </c>
+      <c r="R66">
+        <v>62.155504364900594</v>
+      </c>
+      <c r="S66">
+        <v>17.999392381</v>
       </c>
     </row>
   </sheetData>

</xml_diff>